<commit_message>
feat(F-NAR-019): ATOM-COL.ECO.002-09 Le poisson orange de Mila
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-COL.ECO.002-09.xlsx
+++ b/stories/arbres/ATOM-COL.ECO.002-09.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Le poisson derrière la plante</t>
+          <t>Le poisson orange de Mila</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>cour à l'arrosoir, puis classe au bocal</t>
+          <t>cuisine à la vitre embuée, classe au bocal, puis table</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Mila, papa, maman, maîtresse</t>
+          <t>Mila, papa, maman</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Mila veut revoir le poisson orange derrière la plante. Le mot est déjà là. Elle lève la main, elle attend, puis elle parle.</t>
+          <t>Mila veut dire le poisson orange. Un éclat de poisson brille sur l'écaille. Elle coupe papa : les mots se perdent. À l'école, une voix trop près ; elle coupe, trop vite. Elle refuse de foncer, attend, raconte. Merci vécu. L'éclat de poisson tient l'orange.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>L'arrosoir de la cour a une goutte au bec. La goutte tombe sur la dalle. Un petit serpent d'eau brille, puis s'arrête. Le yaourt de Mila a un fil de miel. Le miel fait un pont, tu vois ? Il est tout doré. Tes bottes rouges attendent sur le paillasson. Elles sont un peu froides. On les enfile. Une. Puis l'autre. Le crayon bleu est derrière ton oreille. Tu l'as senti ? Oui. Il est lisse. Tu voulais revoir le poisson, ce matin. Celui qui se cache. Derrière la plante. Tu le raconteras, si tu veux. Dehors, le brouillard sent l'herbe mouillée. Les bottes font un bruit mou sur le chemin. On tient la main. Le chemin est encore gris. Dans la classe, des poissons en papier pendent. Ils bougent un peu, tout doucement. Un bocal rond brille près de la fenêtre. Le tapis rond est à ta place, Mila. Au revoir. On revient te chercher. Au revoir, maman. Tu poses le sac près du mur. En ce moment, Mila s'assoit sur le tapis rond. Le crayon bleu reste derrière son oreille. Le poisson du bocal fait un petit tour. Il passe derrière la plante verte. Il est encore là. Bonjour. Bonjour. Qui a vu quelque chose qui nage ? Mila a une idée. Le poisson orange derrière la plante. Le mot est déjà là. Elle avance un peu les lèvres. La maîtresse verse encore des graines dans le bocal. Les graines font un tout petit bruit.</t>
+          <t>La vitre de la cuisine est embuée. Le blanc est tiède sous la paume. Mila dessine une petite maison du bout du doigt. Une goutte glisse sur le toit dessiné. Elle a une fenêtre ronde ! Tu as fait le toit, toi ? Oui, et une porte. À côté, Mila dessine un poisson. Le poisson est petit, un peu tordu. Sur une écaille, un éclat de poisson brille. Il brille, papa ! Tu le vois, toi ? Oui, près de la queue. Ça sent le lait tiède, près du bol. Une fumée fine danse au-dessus. Le poisson est orange, dans ma tête. Je veux le dire à l'école. On part après le bol ? Maintenant ! En ce moment, Mila coupe la phrase de papa. Il a une queue, près du toit ! Les deux voix se cognent. Tu disais, Mila ? Le poisson. Personne n'a la phrase entière. Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Papa s'accroupit à la même hauteur. Tu veux parler, ou regarder la goutte ? Parler. Tes bottes rouges attendent sur le paillasson. Les bottes sont un peu froides. On les enfile ? Oui. Une. Puis l'autre. Le crayon bleu est dans ta poche. Tu l'as senti ? Oui. Il est lisse. Dehors, le brouillard sent l'herbe mouillée. Les bottes font un bruit mou sur le chemin. On tient la main ? Oui, papa. Au revoir, Mila. Au revoir, maman. Plus tard, l'école sent la craie. Dans la classe, des poissons en papier pendent. Ils bougent un peu, au plafond. Un bocal rond brille près du mur. Bonjour. Bonjour, maîtresse. Mila s'assoit sur le tapis rond. Le tapis est un peu frais sous les genoux. Le poisson du bocal fait un petit tour. Il est orange, comme le dessin. C'est le même ! Les mots lui chatouillent la bouche. Elle veut le dire, ce poisson, maintenant. Une voix s'approche, trop près. La voix veut le poisson, elle aussi. Attends, je dois parler ! Ses mots se cognent à la voix. Mila referme la bouche. Les mains restent à plat sur ses genoux. Je veux parler du poisson orange.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>L'arrosoir de la cour a une goutte au bec. La goutte tombe sur la dalle. Un petit serpent d'eau brille, puis s'arrête. Le yaourt de Mila a un fil de miel. Le miel fait un pont, tu vois ? Il est tout doré. Tes bottes rouges attendent sur le paillasson. Elles sont un peu froides. On les enfile. Une. Puis l'autre. Le crayon bleu est derrière ton oreille. Tu l'as senti ? Oui. Il est lisse. Tu voulais revoir le poisson, ce matin. Celui qui se cache. Derrière la plante. Tu le raconteras, si tu veux. Dehors, le brouillard sent l'herbe mouillée. Les bottes font un bruit mou sur le chemin. On tient la main. Le chemin est encore gris. Dans la classe, des poissons en papier pendent. Ils bougent un peu, tout doucement. Un bocal rond brille près de la fenêtre. Le tapis rond est à ta place, Mila. Au revoir. On revient te chercher. Au revoir, maman. Tu poses le sac près du mur. En ce moment, Mila s'assoit sur le tapis rond. Le crayon bleu reste derrière son oreille. Le poisson du bocal fait un petit tour. Il passe derrière la plante verte. Il est encore là. Bonjour. Bonjour. Qui a vu quelque chose qui nage ? Mila a une idée. Le poisson orange derrière la plante. Le mot est déjà là. Elle avance un peu les lèvres. La maîtresse verse encore des graines dans le bocal. Les graines font un tout petit bruit.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La vitre de la cuisine est embuée. Le blanc est tiède sous la paume. Mila dessine une petite maison du bout du doigt. Une goutte glisse sur le toit dessiné. Elle a une fenêtre ronde ! Tu as fait le toit, toi ? Oui, et une porte. À côté, Mila dessine un poisson. Le poisson est petit, un peu tordu. Sur une écaille, un &lt;emphasis level="moderate"&gt;éclat de poisson&lt;/emphasis&gt; brille. Il brille, papa ! Tu le vois, toi ? Oui, près de la queue. Ça sent le lait tiède, près du bol. Une fumée fine danse au-dessus. Le poisson est orange, dans ma tête. Je veux le dire à l'école. On part après le bol ? Maintenant ! En ce moment, Mila coupe la phrase de papa. Il a une queue, près du toit ! Les deux voix se cognent. Tu disais, Mila ? Le poisson. Personne n'a la phrase entière. Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Papa s'accroupit à la même hauteur. Tu veux parler, ou regarder la goutte ? Parler. Tes bottes rouges attendent sur le paillasson. Les bottes sont un peu froides. On les enfile ? Oui. Une. Puis l'autre. Le crayon bleu est dans ta poche. Tu l'as senti ? Oui. Il est lisse. Dehors, le brouillard sent l'herbe mouillée. Les bottes font un bruit mou sur le chemin. On tient la main ? Oui, papa. Au revoir, Mila. Au revoir, maman. Plus tard, l'école sent la craie. Dans la classe, des poissons en papier pendent. Ils bougent un peu, au plafond. Un bocal rond brille près du mur. Bonjour. Bonjour, maîtresse. Mila s'assoit sur le tapis rond. Le tapis est un peu frais sous les genoux. Le poisson du bocal fait un petit tour. Il est orange, comme le dessin. C'est le même ! Les mots lui chatouillent la bouche. Elle veut le dire, ce poisson, maintenant. Une voix s'approche, trop près. La voix veut le poisson, elle aussi. Attends, je dois parler ! Ses mots se cognent à la voix. Mila referme la bouche. Les mains restent à plat sur ses genoux. Je veux parler du poisson orange.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Anaïs arrive en classe avec maman. Maman dit au revoir. Anaïs s'assoit sur le tapis. La maîtresse pose une question. Anaïs a une idée. Elle lève la main. Il faut &lt;emphasis&gt;attendre&lt;/emphasis&gt;. Un camarade parle d'abord. Anaïs attend encore. Puis la maîtresse dit : Anaïs, c'est ton tour. Anaïs parle. Elle dit : le chat est gris. La maîtresse sourit. Plus tard, Anaïs a encore une idée. Elle lève la main. Elle attend. Puis elle peut parler. Le soir, maman demande. Anaïs dit : j'ai levé la main. J'ai su attendre. Puis parler, c'était mon tour. [pause]</t>
+          <t>La vitre de la cuisine est embuée. Le blanc est tiède sous la paume. Mila dessine une petite maison du bout du doigt. Une goutte glisse sur le toit dessiné. Elle a une fenêtre ronde ! Tu as fait le toit, toi ? Oui, et une porte. À côté, Mila dessine un poisson. Le poisson est petit, un peu tordu. Sur une écaille, un &lt;emphasis&gt;éclat de poisson&lt;/emphasis&gt; brille. Il brille, papa ! Tu le vois, toi ? Oui, près de la queue. Ça sent le lait tiède, près du bol. Une fumée fine danse au-dessus. Le poisson est orange, dans ma tête. Je veux le dire à l'école. On part après le bol ? Maintenant ! En ce moment, Mila coupe la phrase de papa. Il a une queue, près du toit ! Les deux voix se cognent. Tu disais, Mila ? Le poisson. Personne n'a la phrase entière. Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Papa s'accroupit à la même hauteur. Tu veux parler, ou regarder la goutte ? Parler. Tes bottes rouges attendent sur le paillasson. Les bottes sont un peu froides. On les enfile ? Oui. Une. Puis l'autre. Le crayon bleu est dans ta poche. Tu l'as senti ? Oui. Il est lisse. Dehors, le brouillard sent l'herbe mouillée. Les bottes font un bruit mou sur le chemin. On tient la main ? Oui, papa. Au revoir, Mila. Au revoir, maman. Plus tard, l'école sent la craie. Dans la classe, des poissons en papier pendent. Ils bougent un peu, au plafond. Un bocal rond brille près du mur. Bonjour. Bonjour, maîtresse. Mila s'assoit sur le tapis rond. Le tapis est un peu frais sous les genoux. Le poisson du bocal fait un petit tour. Il est orange, comme le dessin. C'est le même ! Les mots lui chatouillent la bouche. Elle veut le dire, ce poisson, maintenant. Une voix s'approche, trop près. La voix veut le poisson, elle aussi. Attends, je dois parler ! Ses mots se cognent à la voix. Mila referme la bouche. Les mains restent à plat sur ses genoux. Je veux parler du poisson orange. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,7 +1246,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1254,10 +1254,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.18</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>attendre</t>
+          <t>éclat de poisson</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1326,59 +1326,84 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience_curieuse; intensite=2; destinataire=enfant; sous_texte=l_eclat_de_poisson_sur_l_ecaille; tempo=naturel; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|L'arrosoir de la cour a une goutte au bec.
-narrateur|La goutte tombe sur la dalle.
-narrateur|Un petit serpent d'eau brille, puis s'arrête.
-narrateur|Le yaourt de Mila a un fil de miel.
-maman|Le miel fait un pont, tu vois ?
-enfant-f|Il est tout doré.
-papa|Tes bottes rouges attendent sur le paillasson.
-papa|Elles sont un peu froides.
-enfant-f|On les enfile.
+          <t>narrateur|La vitre de la cuisine est embuée.
+narrateur|Le blanc est tiède sous la paume.
+narrateur|Mila dessine une petite maison du bout du doigt.
+narrateur|Une goutte glisse sur le toit dessiné.
+enfant-f|Elle a une fenêtre ronde !
+maman|Tu as fait le toit, toi ?
+enfant-f|Oui, et une porte.
+narrateur|À côté, Mila dessine un poisson.
+narrateur|Le poisson est petit, un peu tordu.
+narrateur|Sur une écaille, un éclat de poisson brille.
+enfant-f|Il brille, papa !
+papa|Tu le vois, toi ?
+enfant-f|Oui, près de la queue.
+narrateur|Ça sent le lait tiède, près du bol.
+narrateur|Une fumée fine danse au-dessus.
+enfant-f|Le poisson est orange, dans ma tête.
+enfant-f|Je veux le dire à l'école.
+papa|On part après le bol ?
+enfant-f|Maintenant !
+narrateur|En ce moment, Mila coupe la phrase de papa.
+enfant-f|Il a une queue, près du toit !
+narrateur|Les deux voix se cognent.
+papa|Tu disais, Mila ?
+enfant-f|Le poisson.
+narrateur|Personne n'a la phrase entière.
+narrateur|Le sourire de Mila disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|Papa s'accroupit à la même hauteur.
+papa|Tu veux parler, ou regarder la goutte ?
+enfant-f|Parler.
+maman|Tes bottes rouges attendent sur le paillasson.
+narrateur|Les bottes sont un peu froides.
+papa|On les enfile ?
+enfant-f|Oui.
 papa|Une.
 papa|Puis l'autre.
-maman|Le crayon bleu est derrière ton oreille.
+maman|Le crayon bleu est dans ta poche.
 maman|Tu l'as senti ?
 enfant-f|Oui.
 enfant-f|Il est lisse.
-papa|Tu voulais revoir le poisson, ce matin.
-enfant-f|Celui qui se cache.
-enfant-f|Derrière la plante.
-maman|Tu le raconteras, si tu veux.
 narrateur|Dehors, le brouillard sent l'herbe mouillée.
 narrateur|Les bottes font un bruit mou sur le chemin.
-papa|On tient la main.
-papa|Le chemin est encore gris.
+papa|On tient la main ?
+enfant-f|Oui, papa.
+maman|Au revoir, Mila.
+enfant-f|Au revoir, maman.
+narrateur|Plus tard, l'école sent la craie.
 narrateur|Dans la classe, des poissons en papier pendent.
-narrateur|Ils bougent un peu, tout doucement.
-narrateur|Un bocal rond brille près de la fenêtre.
-maman|Le tapis rond est à ta place, Mila.
-maman|Au revoir.
-maman|On revient te chercher.
-enfant-f|Au revoir, maman.
-papa|Tu poses le sac près du mur.
-narrateur|En ce moment, Mila s'assoit sur le tapis rond.
-narrateur|Le crayon bleu reste derrière son oreille.
+narrateur|Ils bougent un peu, au plafond.
+narrateur|Un bocal rond brille près du mur.
+maitresse|Bonjour.
+enfant-f|Bonjour, maîtresse.
+narrateur|Mila s'assoit sur le tapis rond.
+narrateur|Le tapis est un peu frais sous les genoux.
 narrateur|Le poisson du bocal fait un petit tour.
-narrateur|Il passe derrière la plante verte.
-enfant-f|Il est encore là.
-maitresse|Bonjour.
-enfant-f|Bonjour.
-maitresse|Qui a vu quelque chose qui nage ?
-narrateur|Mila a une idée.
-narrateur|Le poisson orange derrière la plante.
-narrateur|Le mot est déjà là.
-narrateur|Elle avance un peu les lèvres.
-narrateur|La maîtresse verse encore des graines dans le bocal.
-narrateur|Les graines font un tout petit bruit.</t>
+narrateur|Il est orange, comme le dessin.
+enfant-f|C'est le même !
+narrateur|Les mots lui chatouillent la bouche.
+narrateur|Elle veut le dire, ce poisson, maintenant.
+narrateur|Une voix s'approche, trop près.
+narrateur|La voix veut le poisson, elle aussi.
+enfant-f|Attends, je dois parler !
+narrateur|Ses mots se cognent à la voix.
+narrateur|Mila referme la bouche.
+narrateur|Les mains restent à plat sur ses genoux.
+enfant-f|Je veux parler du poisson orange.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>eau,pas</t>
+          <t>pas,eau</t>
         </is>
       </c>
     </row>
@@ -1410,12 +1435,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Mila veut parler. Que fait-elle d'abord ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Mila veut parler. Que fait-elle &lt;emphasis level="moderate"&gt;d'abord&lt;/emphasis&gt; ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Anaïs veut parler. Que fait-elle d'abord ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Mila veut parler. Que fait-elle &lt;emphasis&gt;d'abord&lt;/emphasis&gt; ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1440,7 +1465,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Elle lève la main et elle attend. Que fait Mila ?</t>
+          <t>Personne ne l'entend. Que fait Mila d'abord ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1478,7 +1503,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1489,7 +1514,7 @@
         <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.3</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1504,34 +1529,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>d'abord</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1546,17 +1575,17 @@
         <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=elle_attend_avant_de_parler; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1589,17 +1618,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Mila lève la main. Elle attend, la main haute. Le poisson passe encore derrière la plante. Mila le suit des yeux. Sa main ne descend pas. Mila, c'est toi. Tu peux parler. Le poisson du bocal est orange. Il se cache derrière la plante. Il nage tout doucement. Derrière la plante, oui. On voit juste sa queue. Merci, Mila. Plus tard, Mila a encore une idée. Les poissons en papier bougent au plafond. Elle lève la main. Elle attend. Mila, c'est encore toi. Les poissons en papier nagent aussi, un peu. Oui. Le crayon bleu glisse dans sa main.</t>
+          <t>Mila lève la main. Sa main reste en l'air. Les doigts tremblent un peu. Une autre voix parle d'abord. On entend parler d'une barque en papier. Mila garde la main levée. Mila ? Mila parle. Le poisson du bocal est orange. Comme le dessin de la maison. Les mots arrivent entiers, cette fois. Sur le flanc, l'éclat de poisson tient. Le soir, les assiettes sont chaudes. Ça sent le gratin. La nappe a des petits carreaux. Alors, Mila ? Mila sent l'envie revenir. Elle lève la main, même à table. Papa écoute maman d'abord. Le gratin est prêt. Mila attend que le silence arrive. Elle pose l'autre main sur la nappe. Mila, c'est toi. Le poisson de l'école est le même. Il nage dans le bocal. Merci de nous le dire, Mila. Papa a entendu toute la phrase. Le ventre de Mila se desserre. Tu as soif ? Un peu. Mila prend une gorgée. L'eau chante contre le verre. C'est frais.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Mila lève la main. Elle attend, la main haute. Le poisson passe encore derrière la plante. Mila le suit des yeux. Sa main ne descend pas. Mila, c'est toi. Tu peux parler. Le poisson du bocal est orange. Il se cache derrière la plante. Il nage tout doucement. Derrière la plante, oui. On voit juste sa queue. Merci, Mila. Plus tard, Mila a encore une idée. Les poissons en papier bougent au plafond. Elle lève la main. Elle attend. Mila, c'est encore toi. Les poissons en papier nagent aussi, un peu. Oui. Le crayon bleu glisse dans sa main.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Mila lève la main. Sa main reste en l'air. Les doigts tremblent un peu. Une autre voix parle d'abord. On entend parler d'une barque en papier. Mila garde la main levée. Mila ? Mila parle. Le poisson du bocal est orange. Comme le dessin de la maison. Les mots arrivent entiers, cette fois. Sur le flanc, l'&lt;emphasis level="moderate"&gt;éclat de poisson&lt;/emphasis&gt; tient. Le soir, les assiettes sont chaudes. Ça sent le gratin. La nappe a des petits carreaux. Alors, Mila ? Mila sent l'envie revenir. Elle lève la main, même à table. Papa écoute maman d'abord. Le gratin est prêt. Mila attend que le silence arrive. Elle pose l'autre main sur la nappe. Mila, c'est toi. Le poisson de l'école est le même. Il nage dans le bocal. Merci de nous le dire, Mila. Papa a entendu toute la phrase. Le ventre de Mila se desserre. Tu as soif ? Un peu. Mila prend une gorgée. L'eau chante contre le verre. C'est frais.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Anaïs a levé la main. Elle a attendu. &lt;emphasis&gt;puis&lt;/emphasis&gt; parler, c'était son tour. [pause]</t>
+          <t>Mila lève la main. Sa main reste en l'air. Les doigts tremblent un peu. Une autre voix parle d'abord. On entend parler d'une barque en papier. Mila garde la main levée. Mila ? Mila parle. Le poisson du bocal est orange. Comme le dessin de la maison. Les mots arrivent entiers, cette fois. Sur le flanc, l'&lt;emphasis&gt;éclat de poisson&lt;/emphasis&gt; tient. Le soir, les assiettes sont chaudes. Ça sent le gratin. La nappe a des petits carreaux. Alors, Mila ? Mila sent l'envie revenir. Elle lève la main, même à table. Papa écoute maman d'abord. Le gratin est prêt. Mila attend que le silence arrive. Elle pose l'autre main sur la nappe. Mila, c'est toi. Le poisson de l'école est le même. Il nage dans le bocal. Merci de nous le dire, Mila. Papa a entendu toute la phrase. Le ventre de Mila se desserre. Tu as soif ? Un peu. Mila prend une gorgée. L'eau chante contre le verre. C'est frais. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1646,7 +1675,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1654,10 +1683,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.18</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1680,30 +1709,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>puis</t>
+          <t>éclat de poisson</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1712,10 +1741,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1728,32 +1757,44 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=elle_attend_puis_on_l_entend; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
           <t>narrateur|Mila lève la main.
-narrateur|Elle attend, la main haute.
-narrateur|Le poisson passe encore derrière la plante.
-narrateur|Mila le suit des yeux.
-narrateur|Sa main ne descend pas.
-maitresse|Mila, c'est toi.
-maitresse|Tu peux parler.
+narrateur|Sa main reste en l'air.
+narrateur|Les doigts tremblent un peu.
+narrateur|Une autre voix parle d'abord.
+narrateur|On entend parler d'une barque en papier.
+narrateur|Mila garde la main levée.
+maitresse|Mila ?
+narrateur|Mila parle.
 enfant-f|Le poisson du bocal est orange.
-enfant-f|Il se cache derrière la plante.
-enfant-f|Il nage tout doucement.
-maitresse|Derrière la plante, oui.
-enfant-f|On voit juste sa queue.
-maitresse|Merci, Mila.
-narrateur|Plus tard, Mila a encore une idée.
-narrateur|Les poissons en papier bougent au plafond.
-narrateur|Elle lève la main.
-narrateur|Elle attend.
-maitresse|Mila, c'est encore toi.
-enfant-f|Les poissons en papier nagent aussi, un peu.
-maitresse|Oui.
-narrateur|Le crayon bleu glisse dans sa main.</t>
+enfant-f|Comme le dessin de la maison.
+narrateur|Les mots arrivent entiers, cette fois.
+narrateur|Sur le flanc, l'éclat de poisson tient.
+narrateur|Le soir, les assiettes sont chaudes.
+narrateur|Ça sent le gratin.
+narrateur|La nappe a des petits carreaux.
+papa|Alors, Mila ?
+narrateur|Mila sent l'envie revenir.
+narrateur|Elle lève la main, même à table.
+narrateur|Papa écoute maman d'abord.
+maman|Le gratin est prêt.
+narrateur|Mila attend que le silence arrive.
+narrateur|Elle pose l'autre main sur la nappe.
+papa|Mila, c'est toi.
+enfant-f|Le poisson de l'école est le même.
+enfant-f|Il nage dans le bocal.
+maman|Merci de nous le dire, Mila.
+narrateur|Papa a entendu toute la phrase.
+narrateur|Le ventre de Mila se desserre.
+papa|Tu as soif ?
+enfant-f|Un peu.
+narrateur|Mila prend une gorgée.
+narrateur|L'eau chante contre le verre.
+enfant-f|C'est frais.</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr">
@@ -1785,17 +1826,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, Mila range son cartable. Le crayon bleu est encore dans sa poche. La porte s'ouvre. Tu as passé un bon moment ? Le poisson était derrière la plante. J'ai parlé de lui. Il était orange ? Oui. On voyait sa queue. On rentre. Le brouillard est parti. La vitre de la cuisine est sèche. Mila pose le crayon bleu sur la table. Je le dessine. La plante, aussi ? Oui. Et sa queue. Je te tiens la feuille.</t>
+          <t>Mila glisse de la chaise. Le poisson, je le montre ! Elle court vers la vitre de la cuisine. Elle frotte d'un grand geste. La maison du doigt disparaît. L'éclat de poisson n'est plus là. Il est parti ! Le sourire tremble. Tu le cherches ? Oui. Mila refuse de foncer. Elle reste près de la vitre. Personne ne parle. Ses doigts attendent sur le bois. Elle souffle sur le verre. Un rideau blanc revient, minuscule. Elle dessine la maison, sans se presser. Puis le poisson, près du toit. Comme ce matin ! Tu le vois, toi ? Mila pose un doigt, sans frotter. L'éclat de poisson saute près de la queue. Il est revenu. Il m'a attendue. La table garde le gratin.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, Mila range son cartable. Le crayon bleu est encore dans sa poche. La porte s'ouvre. Tu as passé un bon moment ? Le poisson était derrière la plante. J'ai parlé de lui. Il était orange ? Oui. On voyait sa queue. On rentre. Le brouillard est parti. La vitre de la cuisine est sèche. Mila pose le crayon bleu sur la table. Je le dessine. La plante, aussi ? Oui. Et sa queue. Je te tiens la feuille.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Mila glisse de la chaise. Le poisson, je le montre ! Elle court vers la vitre de la cuisine. Elle frotte d'un grand geste. La maison du doigt disparaît. L'&lt;emphasis level="moderate"&gt;éclat de poisson&lt;/emphasis&gt; n'est plus là. Il est parti ! Le sourire tremble. Tu le cherches ? Oui. Mila refuse de foncer. Elle reste près de la vitre. Personne ne parle. Ses doigts attendent sur le bois. Elle souffle sur le verre. Un rideau blanc revient, minuscule. Elle dessine la maison, sans se presser. Puis le poisson, près du toit. Comme ce matin ! Tu le vois, toi ? Mila pose un doigt, sans frotter. L'éclat de poisson saute près de la queue. Il est revenu. Il m'a attendue. La table garde le gratin.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Anaïs range son cartable. Maman l'attend à la porte. [pause]</t>
+          <t>&lt;low-pitch&gt;Mila glisse de la chaise. Le poisson, je le montre ! Elle court vers la vitre de la cuisine. Elle frotte d'un grand geste. La maison du doigt disparaît. L'&lt;emphasis&gt;éclat de poisson&lt;/emphasis&gt; n'est plus là. Il est parti ! Le sourire tremble. Tu le cherches ? Oui. Mila refuse de foncer. Elle reste près de la vitre. Personne ne parle. Ses doigts attendent sur le bois. Elle souffle sur le verre. Un rideau blanc revient, minuscule. Elle dessine la maison, sans se presser. Puis le poisson, près du toit. Comme ce matin ! Tu le vois, toi ? Mila pose un doigt, sans frotter. L'éclat de poisson saute près de la queue. Il est revenu. Il m'a attendue. La table garde le gratin.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1842,7 +1883,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1850,22 +1891,26 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="AB5" s="2" t="n">
         <v>1.18</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AE5" s="2" t="inlineStr"/>
+          <t>-2st</t>
+        </is>
+      </c>
+      <c r="AE5" s="2" t="inlineStr">
+        <is>
+          <t>low-pitch</t>
+        </is>
+      </c>
       <c r="AF5" s="2" t="inlineStr">
         <is>
           <t>medium</t>
@@ -1874,28 +1919,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat de poisson</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>520</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>300</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>tense</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1904,41 +1953,52 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
       </c>
       <c r="AT5" s="2" t="n">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=obstacle; intention=alerter_sans_effrayer; emotion=deux_envies_qui_se_heurtent; intensite=2; destinataire=enfant; sous_texte=elle_refuse_de_foncer_retrouve_l_eclat_de_poisson; tempo=resserré; sourire=aucun; respiration=retenue</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Plus tard, Mila range son cartable.
-narrateur|Le crayon bleu est encore dans sa poche.
-narrateur|La porte s'ouvre.
-maman|Tu as passé un bon moment ?
-enfant-f|Le poisson était derrière la plante.
-enfant-f|J'ai parlé de lui.
-papa|Il était orange ?
+          <t>narrateur|Mila glisse de la chaise.
+enfant-f|Le poisson, je le montre !
+narrateur|Elle court vers la vitre de la cuisine.
+narrateur|Elle frotte d'un grand geste.
+narrateur|La maison du doigt disparaît.
+narrateur|L'éclat de poisson n'est plus là.
+enfant-f|Il est parti !
+narrateur|Le sourire tremble.
+papa|Tu le cherches ?
 enfant-f|Oui.
-enfant-f|On voyait sa queue.
-maman|On rentre.
-papa|Le brouillard est parti.
-narrateur|La vitre de la cuisine est sèche.
-narrateur|Mila pose le crayon bleu sur la table.
-enfant-f|Je le dessine.
-maman|La plante, aussi ?
-enfant-f|Oui.
-enfant-f|Et sa queue.
-papa|Je te tiens la feuille.</t>
+narrateur|Mila refuse de foncer.
+narrateur|Elle reste près de la vitre.
+narrateur|Personne ne parle.
+narrateur|Ses doigts attendent sur le bois.
+narrateur|Elle souffle sur le verre.
+narrateur|Un rideau blanc revient, minuscule.
+narrateur|Elle dessine la maison, sans se presser.
+narrateur|Puis le poisson, près du toit.
+enfant-f|Comme ce matin !
+maman|Tu le vois, toi ?
+narrateur|Mila pose un doigt, sans frotter.
+narrateur|L'éclat de poisson saute près de la queue.
+papa|Il est revenu.
+enfant-f|Il m'a attendue.
+narrateur|La table garde le gratin.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
@@ -1970,17 +2030,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le poisson orange est sur la feuille. La plante aussi, un peu de travers. On voit bien sa queue. Bonne soirée, ma grande.</t>
+          <t>Maman souffle un peu sur la vitre. Le poisson orange les regarde. C'est lui. On reste un peu ? Oui, maman. Mila serre le bol contre elle. Le lait n'est plus tiède. On se dit bonne nuit dans un moment ? Oui, papa. Les bottes rouges sèchent sur le paillasson. Il est là. On le garde des yeux ? Oui. L'éclat de poisson tient l'orange.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le poisson orange est sur la feuille. La plante aussi, un peu de travers. On voit bien sa queue. Bonne soirée, ma grande.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Maman souffle un peu sur la vitre. Le poisson orange les regarde. C'est lui. On reste un peu ? Oui, maman. Mila serre le bol contre elle. Le lait n'est plus tiède. On se dit bonne nuit dans un moment ? Oui, papa. Les bottes rouges sèchent sur le paillasson. Il est là. On le garde des yeux ? Oui. L'&lt;emphasis level="moderate"&gt;éclat de poisson&lt;/emphasis&gt; tient l'orange.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Maman souffle un peu sur la vitre. Le poisson orange les regarde. C'est lui. On reste un peu ? Oui, maman. Mila serre le bol contre elle. Le lait n'est plus tiède. On se dit bonne nuit dans un moment ? Oui, papa. Les bottes rouges sèchent sur le paillasson. Il est là. On le garde des yeux ? Oui. L'&lt;emphasis&gt;éclat de poisson&lt;/emphasis&gt; tient l'orange.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2027,7 +2087,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2035,10 +2095,10 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.26</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2047,12 +2107,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2061,17 +2121,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de poisson</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2080,11 +2144,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2093,27 +2157,41 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_de_poisson_tient_l_orange; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|Le poisson orange est sur la feuille.
-narrateur|La plante aussi, un peu de travers.
-papa|On voit bien sa queue.
-maman|Bonne soirée, ma grande.</t>
+          <t>narrateur|Maman souffle un peu sur la vitre.
+narrateur|Le poisson orange les regarde.
+enfant-f|C'est lui.
+maman|On reste un peu ?
+enfant-f|Oui, maman.
+narrateur|Mila serre le bol contre elle.
+narrateur|Le lait n'est plus tiède.
+papa|On se dit bonne nuit dans un moment ?
+enfant-f|Oui, papa.
+narrateur|Les bottes rouges sèchent sur le paillasson.
+enfant-f|Il est là.
+maman|On le garde des yeux ?
+enfant-f|Oui.
+narrateur|L'éclat de poisson tient l'orange.</t>
         </is>
       </c>
     </row>
@@ -2134,7 +2212,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2219,6 +2297,13 @@
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>